<commit_message>
update menambah kolom baru nama inspeksi
</commit_message>
<xml_diff>
--- a/backend/data/reports/riwayat_hasil_ndt.xlsx
+++ b/backend/data/reports/riwayat_hasil_ndt.xlsx
@@ -440,21 +440,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,12 +483,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Keliling P (mm)</t>
+          <t>Luas Babbit (mm2)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Luas Babbit (mm2)</t>
+          <t>Luas Zone A (mm2)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -495,37 +498,52 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Luas Zone A (mm2)</t>
+          <t>Unbond Zone A (mm2)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Total Unbond (mm2)</t>
+          <t>% Unbond Zone A</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Luas Bond (mm2)</t>
+          <t>Status Zone A</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Persen Unbond (%)</t>
+          <t>Unbond Zone C (mm2)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>% Unbond Zone C</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Status Zone C</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Status Akhir</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Inspector</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -533,43 +551,58 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>Zone C</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>565.49</v>
+        <v>57114.15</v>
       </c>
       <c r="F2" t="n">
-        <v>84823</v>
+        <v>30824.33</v>
       </c>
       <c r="G2" t="n">
-        <v>51548.67</v>
+        <v>26289.82</v>
       </c>
       <c r="H2" t="n">
-        <v>33274.33</v>
+        <v>11733</v>
       </c>
       <c r="I2" t="n">
-        <v>7270</v>
-      </c>
-      <c r="J2" t="n">
-        <v>44278.67</v>
+        <v>61.46</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
       </c>
       <c r="K2" t="n">
-        <v>16.42</v>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>kahfi</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -577,39 +610,54 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>Zone C</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>565.49</v>
+        <v>57114.15</v>
       </c>
       <c r="F3" t="n">
-        <v>84823</v>
+        <v>30824.33</v>
       </c>
       <c r="G3" t="n">
-        <v>51548.67</v>
+        <v>26289.82</v>
       </c>
       <c r="H3" t="n">
-        <v>33274.33</v>
+        <v>39</v>
       </c>
       <c r="I3" t="n">
-        <v>2720</v>
-      </c>
-      <c r="J3" t="n">
-        <v>48828.67</v>
+        <v>0.13</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
       </c>
       <c r="K3" t="n">
-        <v>5.57</v>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
+        <v>300</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -617,43 +665,58 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>360</v>
+        <v>19</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone D</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>565.49</v>
+        <v>22234.62</v>
       </c>
       <c r="F4" t="n">
-        <v>113097.34</v>
+        <v>36242.26</v>
       </c>
       <c r="G4" t="n">
-        <v>77323</v>
+        <v>-14007.63</v>
       </c>
       <c r="H4" t="n">
-        <v>35774.33</v>
+        <v>525</v>
       </c>
       <c r="I4" t="n">
-        <v>1100</v>
-      </c>
-      <c r="J4" t="n">
-        <v>76223</v>
+        <v>1.47</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
       </c>
       <c r="K4" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>2304</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-14.12</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -661,43 +724,58 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>565.49</v>
+        <v>692.72</v>
       </c>
       <c r="F5" t="n">
-        <v>113097.34</v>
+        <v>199.34</v>
       </c>
       <c r="G5" t="n">
-        <v>77323</v>
+        <v>493.39</v>
       </c>
       <c r="H5" t="n">
-        <v>35774.33</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>665</v>
-      </c>
-      <c r="J5" t="n">
-        <v>76658</v>
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
       </c>
       <c r="K5" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>6371</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-108.39</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -705,43 +783,58 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>565.49</v>
+        <v>692.72</v>
       </c>
       <c r="F6" t="n">
-        <v>113097.34</v>
+        <v>199.34</v>
       </c>
       <c r="G6" t="n">
-        <v>77323</v>
+        <v>493.39</v>
       </c>
       <c r="H6" t="n">
-        <v>35774.33</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>500</v>
-      </c>
-      <c r="J6" t="n">
-        <v>76823</v>
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
       </c>
       <c r="K6" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>6371</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-108.39</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -749,43 +842,58 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>565.49</v>
+        <v>692.72</v>
       </c>
       <c r="F7" t="n">
-        <v>113097.34</v>
+        <v>199.34</v>
       </c>
       <c r="G7" t="n">
-        <v>77323</v>
+        <v>493.39</v>
       </c>
       <c r="H7" t="n">
-        <v>35774.33</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>800</v>
-      </c>
-      <c r="J7" t="n">
-        <v>76523</v>
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
       </c>
       <c r="K7" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>341</v>
+      </c>
+      <c r="L7" t="n">
+        <v>223.78</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -793,81 +901,403 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>565.49</v>
+        <v>692.72</v>
       </c>
       <c r="F8" t="n">
-        <v>113097.34</v>
+        <v>199.34</v>
       </c>
       <c r="G8" t="n">
-        <v>77323</v>
+        <v>493.39</v>
       </c>
       <c r="H8" t="n">
-        <v>35774.33</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>820</v>
-      </c>
-      <c r="J8" t="n">
-        <v>76503</v>
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
       </c>
       <c r="K8" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>341</v>
+      </c>
+      <c r="L8" t="n">
+        <v>223.78</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>49</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1616.35</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2398.45</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-782.1</v>
+      </c>
+      <c r="J9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>360</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>84823</v>
+      </c>
+      <c r="F10" t="n">
+        <v>33274.33</v>
+      </c>
+      <c r="G10" t="n">
+        <v>51548.67</v>
+      </c>
+      <c r="J10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>360</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>84823</v>
+      </c>
+      <c r="F11" t="n">
+        <v>33274.33</v>
+      </c>
+      <c r="G11" t="n">
+        <v>51548.67</v>
+      </c>
+      <c r="J11" s="2" t="n"/>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>360</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F12" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G12" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>360</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F13" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G13" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>360</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F14" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G14" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>360</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F15" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G15" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J15" s="2" t="n"/>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>360</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F16" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G16" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J16" s="2" t="n"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
         <v>1</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>bearing</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C17" t="n">
         <v>360</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Zona A</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>565.49</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="E17" t="n">
         <v>113097.34</v>
       </c>
-      <c r="G9" t="n">
+      <c r="F17" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G17" t="n">
         <v>77323</v>
       </c>
-      <c r="H9" t="n">
-        <v>35774.33</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1100</v>
-      </c>
-      <c r="J9" t="n">
-        <v>76223</v>
-      </c>
-      <c r="K9" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+      <c r="J17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
drawing mapping & export pdf
</commit_message>
<xml_diff>
--- a/backend/data/reports/riwayat_hasil_ndt.xlsx
+++ b/backend/data/reports/riwayat_hasil_ndt.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -539,35 +539,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bearing</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>360</v>
+        <v>42</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Zone C</t>
+          <t>zone W</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>57114.15</v>
+        <v>4024.38</v>
       </c>
       <c r="F2" t="n">
-        <v>30824.33</v>
+        <v>4018.41</v>
       </c>
       <c r="G2" t="n">
-        <v>26289.82</v>
+        <v>5.97</v>
       </c>
       <c r="H2" t="n">
-        <v>11733</v>
+        <v>1683</v>
       </c>
       <c r="I2" t="n">
-        <v>61.46</v>
+        <v>72.06</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -575,14 +575,14 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1920</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>-100.31</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -592,72 +592,72 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>kahfi</t>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bearing</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>360</v>
+        <v>18</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Zone C</t>
+          <t>zone D</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>57114.15</v>
+        <v>424.12</v>
       </c>
       <c r="F3" t="n">
-        <v>30824.33</v>
+        <v>-336.28</v>
       </c>
       <c r="G3" t="n">
-        <v>26289.82</v>
+        <v>760.4</v>
       </c>
       <c r="H3" t="n">
-        <v>39</v>
+        <v>204</v>
       </c>
       <c r="I3" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>-37.76</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>300</v>
+        <v>782</v>
       </c>
       <c r="L3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>-3620.09</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -673,19 +673,19 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>22234.62</v>
+        <v>424.12</v>
       </c>
       <c r="F4" t="n">
-        <v>36242.26</v>
+        <v>-336.28</v>
       </c>
       <c r="G4" t="n">
-        <v>-14007.63</v>
+        <v>760.4</v>
       </c>
       <c r="H4" t="n">
-        <v>525</v>
+        <v>204</v>
       </c>
       <c r="I4" t="n">
-        <v>1.47</v>
+        <v>-37.76</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -693,10 +693,10 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2304</v>
+        <v>782</v>
       </c>
       <c r="L4" t="n">
-        <v>-14.12</v>
+        <v>-3620.09</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -710,35 +710,35 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21</v>
+        <v>360</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>zone a</t>
+          <t>Zone C</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>692.72</v>
+        <v>57114.15</v>
       </c>
       <c r="F5" t="n">
-        <v>199.34</v>
+        <v>12929.73</v>
       </c>
       <c r="G5" t="n">
-        <v>493.39</v>
+        <v>44184.42</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -752,69 +752,69 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>6371</v>
+        <v>231</v>
       </c>
       <c r="L5" t="n">
-        <v>-108.39</v>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
+        <v>0.53</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kahfi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>21</v>
+        <v>360</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>zone a</t>
+          <t>Zone C</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>692.72</v>
+        <v>57114.15</v>
       </c>
       <c r="F6" t="n">
-        <v>199.34</v>
+        <v>30824.33</v>
       </c>
       <c r="G6" t="n">
-        <v>493.39</v>
+        <v>26289.82</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>252</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>0.82</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>6371</v>
+        <v>1113</v>
       </c>
       <c r="L6" t="n">
-        <v>-108.39</v>
+        <v>4.42</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -828,56 +828,56 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>staff1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>360</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>zone a</t>
+          <t>Zone C</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>692.72</v>
+        <v>57114.15</v>
       </c>
       <c r="F7" t="n">
-        <v>199.34</v>
+        <v>30824.33</v>
       </c>
       <c r="G7" t="n">
-        <v>493.39</v>
+        <v>26289.82</v>
       </c>
       <c r="H7" t="n">
+        <v>11733</v>
+      </c>
+      <c r="I7" t="n">
+        <v>61.46</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="I7" t="n">
+      <c r="L7" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>341</v>
-      </c>
-      <c r="L7" t="n">
-        <v>223.78</v>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -887,41 +887,41 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kahfi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>21</v>
+        <v>360</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>zone a</t>
+          <t>Zone C</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>692.72</v>
+        <v>57114.15</v>
       </c>
       <c r="F8" t="n">
-        <v>199.34</v>
+        <v>30824.33</v>
       </c>
       <c r="G8" t="n">
-        <v>493.39</v>
+        <v>26289.82</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
@@ -929,19 +929,19 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="L8" t="n">
-        <v>223.78</v>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
+        <v>1.15</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -952,7 +952,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -960,27 +960,47 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>zone D</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1616.35</v>
+        <v>22234.62</v>
       </c>
       <c r="F9" t="n">
-        <v>2398.45</v>
+        <v>36242.26</v>
       </c>
       <c r="G9" t="n">
-        <v>-782.1</v>
-      </c>
-      <c r="J9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>-14007.63</v>
+      </c>
+      <c r="H9" t="n">
+        <v>525</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>2304</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-14.12</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -991,7 +1011,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -999,24 +1019,44 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>84823</v>
+        <v>692.72</v>
       </c>
       <c r="F10" t="n">
-        <v>33274.33</v>
+        <v>199.34</v>
       </c>
       <c r="G10" t="n">
-        <v>51548.67</v>
-      </c>
-      <c r="J10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
+        <v>493.39</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>6371</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-108.39</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
           <t>REJECT</t>
@@ -1030,7 +1070,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1038,24 +1078,44 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>84823</v>
+        <v>692.72</v>
       </c>
       <c r="F11" t="n">
-        <v>33274.33</v>
+        <v>199.34</v>
       </c>
       <c r="G11" t="n">
-        <v>51548.67</v>
-      </c>
-      <c r="J11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
+        <v>493.39</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>6371</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-108.39</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
           <t>REJECT</t>
@@ -1069,7 +1129,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1077,27 +1137,47 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>113097.34</v>
+        <v>692.72</v>
       </c>
       <c r="F12" t="n">
-        <v>35774.33</v>
+        <v>199.34</v>
       </c>
       <c r="G12" t="n">
-        <v>77323</v>
-      </c>
-      <c r="J12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>493.39</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>341</v>
+      </c>
+      <c r="L12" t="n">
+        <v>223.78</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1108,7 +1188,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1116,27 +1196,47 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>113097.34</v>
+        <v>692.72</v>
       </c>
       <c r="F13" t="n">
-        <v>35774.33</v>
+        <v>199.34</v>
       </c>
       <c r="G13" t="n">
-        <v>77323</v>
-      </c>
-      <c r="J13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+        <v>493.39</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>341</v>
+      </c>
+      <c r="L13" t="n">
+        <v>223.78</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1147,7 +1247,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1155,21 +1255,21 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>360</v>
+        <v>49</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>b</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>113097.34</v>
+        <v>1616.35</v>
       </c>
       <c r="F14" t="n">
-        <v>35774.33</v>
+        <v>2398.45</v>
       </c>
       <c r="G14" t="n">
-        <v>77323</v>
+        <v>-782.1</v>
       </c>
       <c r="J14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
@@ -1186,7 +1286,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1202,19 +1302,19 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>113097.34</v>
+        <v>84823</v>
       </c>
       <c r="F15" t="n">
-        <v>35774.33</v>
+        <v>33274.33</v>
       </c>
       <c r="G15" t="n">
-        <v>77323</v>
+        <v>51548.67</v>
       </c>
       <c r="J15" s="2" t="n"/>
       <c r="M15" s="2" t="n"/>
-      <c r="N15" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1225,7 +1325,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1241,19 +1341,19 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>113097.34</v>
+        <v>84823</v>
       </c>
       <c r="F16" t="n">
-        <v>35774.33</v>
+        <v>33274.33</v>
       </c>
       <c r="G16" t="n">
-        <v>77323</v>
+        <v>51548.67</v>
       </c>
       <c r="J16" s="2" t="n"/>
       <c r="M16" s="2" t="n"/>
-      <c r="N16" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1264,7 +1364,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1296,6 +1396,201 @@
         </is>
       </c>
       <c r="O17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>360</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F18" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G18" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J18" s="2" t="n"/>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>360</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F19" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G19" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>360</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F20" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G20" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>360</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F21" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G21" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J21" s="2" t="n"/>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>360</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F22" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G22" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
menambahkan input gambar pada form tambah indikasi
</commit_message>
<xml_diff>
--- a/backend/data/reports/riwayat_hasil_ndt.xlsx
+++ b/backend/data/reports/riwayat_hasil_ndt.xlsx
@@ -45,14 +45,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DC2626"/>
-        <bgColor rgb="00DC2626"/>
+        <fgColor rgb="0016A34A"/>
+        <bgColor rgb="0016A34A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0016A34A"/>
-        <bgColor rgb="0016A34A"/>
+        <fgColor rgb="00DC2626"/>
+        <bgColor rgb="00DC2626"/>
       </patternFill>
     </fill>
   </fills>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -458,6 +458,7 @@
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,209 +537,229 @@
           <t>Inspector</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Asal</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>42</v>
+        <v>150</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>zone W</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4024.38</v>
+        <v>23797.56</v>
       </c>
       <c r="F2" t="n">
-        <v>4018.41</v>
+        <v>6391.67</v>
       </c>
       <c r="G2" t="n">
-        <v>5.97</v>
+        <v>17405.89</v>
       </c>
       <c r="H2" t="n">
-        <v>1683</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>72.06</v>
+        <v>0</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>REJECT</t>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1920</v>
+        <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>-100.31</v>
+        <v>0.58</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>REJECT</t>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>REJECT</t>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>PLTA Maninjau</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>zone D</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>424.12</v>
+        <v>15150</v>
       </c>
       <c r="F3" t="n">
-        <v>-336.28</v>
+        <v>4662.16</v>
       </c>
       <c r="G3" t="n">
-        <v>760.4</v>
+        <v>10487.84</v>
       </c>
       <c r="H3" t="n">
-        <v>204</v>
+        <v>2720</v>
       </c>
       <c r="I3" t="n">
-        <v>-37.76</v>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
+        <v>140.05</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>782</v>
+        <v>4550</v>
       </c>
       <c r="L3" t="n">
-        <v>-3620.09</v>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
+        <v>76.63</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>PLTA Maninjau</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>zone D</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>424.12</v>
+        <v>15150</v>
       </c>
       <c r="F4" t="n">
-        <v>-336.28</v>
+        <v>4662.16</v>
       </c>
       <c r="G4" t="n">
-        <v>760.4</v>
+        <v>10487.84</v>
       </c>
       <c r="H4" t="n">
-        <v>204</v>
+        <v>2720</v>
       </c>
       <c r="I4" t="n">
-        <v>-37.76</v>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
+        <v>140.05</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>782</v>
+        <v>4550</v>
       </c>
       <c r="L4" t="n">
-        <v>-3620.09</v>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
+        <v>76.63</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>PLTA Maninjau</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bearing</t>
+          <t>Beearing</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>360</v>
+        <v>150</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Zone C</t>
+          <t>Lower</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>57114.15</v>
+        <v>23797.56</v>
       </c>
       <c r="F5" t="n">
-        <v>12929.73</v>
+        <v>6391.67</v>
       </c>
       <c r="G5" t="n">
-        <v>44184.42</v>
+        <v>17405.89</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -746,23 +767,23 @@
       <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>231</v>
+        <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
+        <v>0.58</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
@@ -770,71 +791,81 @@
       <c r="O5" t="inlineStr">
         <is>
           <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bearing</t>
+          <t>Beearing</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>360</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Zone C</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>57114.15</v>
+        <v>15150</v>
       </c>
       <c r="F6" t="n">
-        <v>30824.33</v>
+        <v>4662.16</v>
       </c>
       <c r="G6" t="n">
-        <v>26289.82</v>
+        <v>10487.84</v>
       </c>
       <c r="H6" t="n">
-        <v>252</v>
+        <v>2720</v>
       </c>
       <c r="I6" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
+        <v>140.05</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>1113</v>
+        <v>4550</v>
       </c>
       <c r="L6" t="n">
-        <v>4.42</v>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
+        <v>76.63</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>staff1</t>
+          <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -842,58 +873,63 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>360</v>
+        <v>17</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Zone C</t>
+          <t>Lower</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>57114.15</v>
+        <v>721</v>
       </c>
       <c r="F7" t="n">
-        <v>30824.33</v>
+        <v>260.84</v>
       </c>
       <c r="G7" t="n">
-        <v>26289.82</v>
+        <v>460.16</v>
       </c>
       <c r="H7" t="n">
-        <v>11733</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>61.46</v>
+        <v>0</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>REJECT</t>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1948</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>-130.93</v>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>kahfi</t>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -901,50 +937,55 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>360</v>
+        <v>65</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Zone C</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>57114.15</v>
+        <v>10822.79</v>
       </c>
       <c r="F8" t="n">
-        <v>30824.33</v>
+        <v>3962.32</v>
       </c>
       <c r="G8" t="n">
-        <v>26289.82</v>
+        <v>6860.47</v>
       </c>
       <c r="H8" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>300</v>
+        <v>1560</v>
       </c>
       <c r="L8" t="n">
-        <v>1.15</v>
+        <v>29.43</v>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -952,7 +993,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -960,50 +1001,55 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19</v>
+        <v>795</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>zone D</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>22234.62</v>
+        <v>427083.81</v>
       </c>
       <c r="F9" t="n">
-        <v>36242.26</v>
+        <v>104131</v>
       </c>
       <c r="G9" t="n">
-        <v>-14007.63</v>
+        <v>322952.81</v>
       </c>
       <c r="H9" t="n">
-        <v>525</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1.47</v>
+        <v>0</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>REJECT</t>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>2304</v>
+        <v>8612</v>
       </c>
       <c r="L9" t="n">
-        <v>-14.12</v>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
+        <v>2.74</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1011,7 +1057,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1019,21 +1065,21 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>21</v>
+        <v>123</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>zone a</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>692.72</v>
+        <v>5989.45</v>
       </c>
       <c r="F10" t="n">
-        <v>199.34</v>
+        <v>1351.65</v>
       </c>
       <c r="G10" t="n">
-        <v>493.39</v>
+        <v>4637.8</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -1041,28 +1087,33 @@
       <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>6371</v>
+        <v>1253</v>
       </c>
       <c r="L10" t="n">
-        <v>-108.39</v>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
+        <v>37.02</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1070,7 +1121,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1078,21 +1129,21 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21</v>
+        <v>123</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>zone a</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>692.72</v>
+        <v>5989.45</v>
       </c>
       <c r="F11" t="n">
-        <v>199.34</v>
+        <v>1351.65</v>
       </c>
       <c r="G11" t="n">
-        <v>493.39</v>
+        <v>4637.8</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1100,28 +1151,33 @@
       <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>6371</v>
+        <v>1253</v>
       </c>
       <c r="L11" t="n">
-        <v>-108.39</v>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
+        <v>37.02</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1129,29 +1185,29 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>21</v>
+        <v>234</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>zone a</t>
+          <t>Lower</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>692.72</v>
+        <v>158788.66</v>
       </c>
       <c r="F12" t="n">
-        <v>199.34</v>
+        <v>61617.57</v>
       </c>
       <c r="G12" t="n">
-        <v>493.39</v>
+        <v>97171.09</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -1159,28 +1215,33 @@
       <c r="I12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>341</v>
+        <v>10620</v>
       </c>
       <c r="L12" t="n">
-        <v>223.78</v>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
+        <v>12.27</v>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1188,7 +1249,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1196,50 +1257,51 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>zone a</t>
-        </is>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>692.72</v>
+        <v>5105.09</v>
       </c>
       <c r="F13" t="n">
-        <v>199.34</v>
+        <v>5748.34</v>
       </c>
       <c r="G13" t="n">
-        <v>493.39</v>
+        <v>-643.26</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>176</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>3.16</v>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>341</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>223.78</v>
+        <v>0</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1247,38 +1309,63 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1616.35</v>
+        <v>15150</v>
       </c>
       <c r="F14" t="n">
-        <v>2398.45</v>
+        <v>4620</v>
       </c>
       <c r="G14" t="n">
-        <v>-782.1</v>
-      </c>
-      <c r="J14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
+        <v>10530</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2720</v>
+      </c>
+      <c r="I14" t="n">
+        <v>143.16</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>4550</v>
+      </c>
+      <c r="L14" t="n">
+        <v>76.09</v>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
+        <is>
+          <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1286,38 +1373,63 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>360</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>84823</v>
+        <v>15135.25</v>
       </c>
       <c r="F15" t="n">
-        <v>33274.33</v>
+        <v>9868.5</v>
       </c>
       <c r="G15" t="n">
-        <v>51548.67</v>
-      </c>
-      <c r="J15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="inlineStr">
+        <v>5266.75</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2720</v>
+      </c>
+      <c r="I15" t="n">
+        <v>38.05</v>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>4550</v>
+      </c>
+      <c r="L15" t="n">
+        <v>634.8099999999999</v>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
+        <is>
+          <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1325,11 +1437,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1337,7 +1449,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1349,14 +1461,39 @@
       <c r="G16" t="n">
         <v>51548.67</v>
       </c>
-      <c r="J16" s="2" t="n"/>
-      <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="H16" t="n">
+        <v>2720</v>
+      </c>
+      <c r="I16" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>4550</v>
+      </c>
+      <c r="L16" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
+        <is>
+          <t>kahfi</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1364,7 +1501,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1372,30 +1509,55 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>360</v>
+        <v>65</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>113097.34</v>
+        <v>5105.09</v>
       </c>
       <c r="F17" t="n">
-        <v>35774.33</v>
+        <v>5105.09</v>
       </c>
       <c r="G17" t="n">
-        <v>77323</v>
-      </c>
-      <c r="J17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>14760</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-152.88</v>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1403,11 +1565,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>Bearing</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1415,26 +1577,51 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>Zone C</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>113097.34</v>
+        <v>57114.15</v>
       </c>
       <c r="F18" t="n">
-        <v>35774.33</v>
+        <v>30824.33</v>
       </c>
       <c r="G18" t="n">
-        <v>77323</v>
-      </c>
-      <c r="J18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="3" t="inlineStr">
+        <v>26289.82</v>
+      </c>
+      <c r="H18" t="n">
+        <v>39</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>300</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1442,7 +1629,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1450,30 +1637,55 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>113097.34</v>
+        <v>692.72</v>
       </c>
       <c r="F19" t="n">
-        <v>35774.33</v>
+        <v>199.34</v>
       </c>
       <c r="G19" t="n">
-        <v>77323</v>
-      </c>
-      <c r="J19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
+        <v>493.39</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>6371</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-108.39</v>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1481,7 +1693,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1489,30 +1701,55 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>360</v>
+        <v>21</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>zone a</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>113097.34</v>
+        <v>692.72</v>
       </c>
       <c r="F20" t="n">
-        <v>35774.33</v>
+        <v>199.34</v>
       </c>
       <c r="G20" t="n">
-        <v>77323</v>
-      </c>
-      <c r="J20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
+        <v>493.39</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>341</v>
+      </c>
+      <c r="L20" t="n">
+        <v>223.78</v>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>ACCEPT</t>
+          <t>REJECT</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1520,7 +1757,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1528,30 +1765,35 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>360</v>
+        <v>49</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Zona A</t>
+          <t>b</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>113097.34</v>
+        <v>1616.35</v>
       </c>
       <c r="F21" t="n">
-        <v>35774.33</v>
+        <v>2398.45</v>
       </c>
       <c r="G21" t="n">
-        <v>77323</v>
-      </c>
-      <c r="J21" s="2" t="n"/>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="3" t="inlineStr">
+        <v>-782.1</v>
+      </c>
+      <c r="J21" s="3" t="n"/>
+      <c r="M21" s="3" t="n"/>
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>ACCEPT</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1559,7 +1801,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1575,22 +1817,335 @@
         </is>
       </c>
       <c r="E22" t="n">
+        <v>84823</v>
+      </c>
+      <c r="F22" t="n">
+        <v>33274.33</v>
+      </c>
+      <c r="G22" t="n">
+        <v>51548.67</v>
+      </c>
+      <c r="J22" s="3" t="n"/>
+      <c r="M22" s="3" t="n"/>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>360</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>84823</v>
+      </c>
+      <c r="F23" t="n">
+        <v>33274.33</v>
+      </c>
+      <c r="G23" t="n">
+        <v>51548.67</v>
+      </c>
+      <c r="J23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>360</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
         <v>113097.34</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F24" t="n">
         <v>35774.33</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G24" t="n">
         <v>77323</v>
       </c>
-      <c r="J22" s="2" t="n"/>
-      <c r="M22" s="2" t="n"/>
-      <c r="N22" s="3" t="inlineStr">
-        <is>
-          <t>ACCEPT</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="J24" s="3" t="n"/>
+      <c r="M24" s="3" t="n"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>360</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F25" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G25" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>360</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F26" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G26" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J26" s="3" t="n"/>
+      <c r="M26" s="3" t="n"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>360</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F27" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G27" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J27" s="3" t="n"/>
+      <c r="M27" s="3" t="n"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>360</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F28" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G28" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J28" s="3" t="n"/>
+      <c r="M28" s="3" t="n"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>360</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Zona A</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>113097.34</v>
+      </c>
+      <c r="F29" t="n">
+        <v>35774.33</v>
+      </c>
+      <c r="G29" t="n">
+        <v>77323</v>
+      </c>
+      <c r="J29" s="3" t="n"/>
+      <c r="M29" s="3" t="n"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>